<commit_message>
notes(gpu-specs): add Kunlunxin P800, M100 and M300
P800 has no official spec page — Kunlunxin lists only the R and K series —
so every spec row is 无. Its official news does confirm the part ships, and
those two posts are cited for the CAICT DeepSeek 671B test and the openEuler
certification. The widely quoted 96 GB / 345 TFLOPS / 2.4 TB/s figures have
no official source and are called out as such.

P900 does not appear anywhere official, so the roadmap parts Baidu did
announce stand in for it: M100 and M300, both 无 throughout, with the
announcement noted in the intro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notes/_research/gpu-hardware-scope.xlsx
+++ b/notes/_research/gpu-hardware-scope.xlsx
@@ -16,16 +16,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intel" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Microsoft" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="寒武纪" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="沐曦" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摩尔线程" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="壁仞" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="海光" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Groq" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cerebras" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="昆仑芯" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="寒武纪" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="沐曦" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摩尔线程" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="壁仞" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="海光" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Groq" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cerebras" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'机型清单'!$A$1:$N$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'机型清单'!$A$1:$N$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -549,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2433,9 +2434,219 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>昆仑芯</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>P800</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>无官方公开参数（仅官方新闻提及型号）</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>无：昆仑芯官网产品信息仅列 R / K 系列，无 P800 规格页</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>XPU</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>NPU</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>量产</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>国产章</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>国产里出货与集群规模最实的一条线：官方新闻确认已通过信通院 DeepSeek 671B 满血版适配、并与 openEuler 完成兼容性互认证</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>官网无规格页，参数全部为「无」；流传的 96 GB / 345 TFLOPS 无官方出处</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>昆仑芯</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>M100</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>无官方公开参数</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>无：昆仑芯官网无 M 系列页面</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>XPU</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>NPU</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>宣布</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>2026 初（计划）</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>国产章附表</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>百度世界大会 2025 公布的第四代，定位大规模推理；用来标注国产路线图的下一跳</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>官网无 M 系列页面，无任何官方参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>昆仑芯</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>M300</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>无官方公开参数</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>无：昆仑芯官网无 M 系列页面</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>XPU</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>NPU</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>宣布</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2027 初（计划）</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>国产章附表</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>同一路线图里面向超大规模多模态训练 / 推理的一代</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>官网无 M 系列页面，无任何官方参数</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N27"/>
-  <conditionalFormatting sqref="M2:M27">
+  <autoFilter ref="A1:N30"/>
+  <conditionalFormatting sqref="M2:M30">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"低"</formula>
     </cfRule>
@@ -2444,10 +2655,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="只能是 P0 / P1 / P2" type="list">
+    <dataValidation sqref="B2:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="只能是 P0 / P1 / P2" type="list">
       <formula1>"P0,P1,P2"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2484,21 +2695,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>寒武纪 · 官方参数</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
+          <t>昆仑芯 · 官方参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>只收厂商白皮书、datasheet、官网规格页与官方博客 / 文档里写明的数；原文没写的一律填「无」，不换算、不由整机反推单卡；稀疏 / 稠密照原文标注。①②③ 对应表底的来源。核对日期 2026-10-26。</t>
@@ -2513,11 +2726,21 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>思元 690</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
+          <t>P800</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>M100</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>M300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>简介（据官方文档）</t>
@@ -2525,7 +2748,17 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>无：寒武纪官网产品页仅列至思元 370（MLU370），未发布思元 690 的规格或白皮书</t>
+          <t>无官方规格：昆仑芯官网「产品信息」只列 R 系列（昆仑芯 2 代、R100、R200、RG800、R480-X8）与 K 系列（昆仑芯 1 代、K100、K200），未发布 P800 的规格页或白皮书 ③；官方新闻确认该型号存在且已规模交付 ①②</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>无：昆仑芯官网未发布 M100 的规格页或白皮书，站内新闻也未出现该型号；型号与定位（面向大规模推理、计划 2026 年初上市）出自 2025-11-13 百度世界大会的公开发布</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>无：昆仑芯官网未发布 M300 的规格页或白皮书，站内新闻也未出现该型号；型号与定位（面向超大规模多模态模型训练与推理、计划 2027 年初上市）出自 2025-11-13 百度世界大会的公开发布</t>
         </is>
       </c>
     </row>
@@ -2540,6 +2773,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -2552,6 +2795,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -2564,6 +2817,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -2576,6 +2839,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -2588,6 +2861,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -2600,6 +2883,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -2612,6 +2905,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -2624,6 +2927,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -2636,6 +2949,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
@@ -2648,6 +2971,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
@@ -2660,6 +2993,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -2672,6 +3015,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -2684,6 +3037,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -2696,6 +3059,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -2708,6 +3081,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -2720,6 +3103,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
@@ -2732,6 +3125,16 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -2744,32 +3147,62 @@
           <t>无</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="104" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
           <t>其他官方指标</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>官方新闻口径：P800 单机 8 卡一体机通过中国信通院 DeepSeek-V3/R1 671B 满血版适配支持性测试，精度与 DeepSeek 技术报告对齐、支持长上下文推理，为首个通过该测试的产品 ①；P800 系列与 openEuler 完成兼容性互认证，七项子测试全部通过 ②</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>官方新闻只写适配与认证结果，未给出显存、算力、带宽、功耗等任何参数，故本列参数全部为「无」；流传的 96 GB HBM、345 TFLOPS FP16、2.4 TB/s 等数字均出自媒体报道，未见官方文档，不予采信</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>本列无任何官方参数。大会路线图只给定位与上市时间，且未见官方文档原文，故不填入参数行</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>本列无任何官方参数。大会路线图只给定位与上市时间，且未见官方文档原文，故不填入参数行</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="76" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
           <t>来源 ①</t>
@@ -2777,18 +3210,80 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>已核查：寒武纪官网产品中心（无思元 690）
-https://www.cambricon.com/</t>
+          <t>官方新闻：昆仑芯 · 首个！昆仑芯 P800 单机 8 卡一体机通过中国信通院 DeepSeek 适配测试（2025-04-17）
+https://www.kunlunxin.com/news/4471.html</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>已核查：昆仑芯官网产品信息（无 M 系列页面）
+https://www.kunlunxin.com/</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>已核查：昆仑芯官网产品信息（无 M 系列页面）
+https://www.kunlunxin.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>来源 ②</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>官方新闻：昆仑芯 · 与 openEuler 完成兼容性互认证（2026-10-23）
+https://www.kunlunxin.com/news/5195.html</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>来源 ③</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>已核查：昆仑芯官网产品信息（仅列 R / K 系列，无 P800 规格页）
+https://www.kunlunxin.com/</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2810,7 +3305,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>沐曦 · 官方参数</t>
+          <t>寒武纪 · 官方参数</t>
         </is>
       </c>
     </row>
@@ -2829,19 +3324,19 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>曦云 C600</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
+          <t>思元 690</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>简介（据官方文档）</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>沐曦基于自主知识产权 GPGPU 架构与国产先进工艺研发的新一代通用 GPU，面向智算中心、通用计算与数据分析；配 MXMACA 软件栈（兼容主流 GPU 生态）</t>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>无：寒武纪官网产品页仅列至思元 370（MLU370），未发布思元 690 的规格或白皮书</t>
         </is>
       </c>
     </row>
@@ -2851,9 +3346,9 @@
           <t>架构</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>自主知识产权 GPGPU 架构（未写代号）</t>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -2863,9 +3358,9 @@
           <t>制程 / 晶体管 / 封装</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>国产先进工艺（未写节点）</t>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -2875,9 +3370,9 @@
           <t>形态 / 散热</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>OAM 2.0 扣卡式模组；风冷 / 液冷</t>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -2889,7 +3384,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>无（官网仅称「超大容量高带宽显存」，支持全链路 ECC）</t>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -3019,9 +3514,9 @@
           <t>Scale-up 互连</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>MetaXLink 互连；MetaXLink-E 接口最高 128 卡超节点</t>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -3043,9 +3538,9 @@
           <t>功耗</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>最大功耗 1000W</t>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -3093,8 +3588,8 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>官网产品页：沐曦 · 曦云C600
-https://www.metax-tech.com/prod.html?cid=107&amp;id=68</t>
+          <t>已核查：寒武纪官网产品中心（无思元 690）
+https://www.cambricon.com/</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3126,7 +3621,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>摩尔线程 · 官方参数</t>
+          <t>沐曦 · 官方参数</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3640,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>MTT S5000</t>
+          <t>曦云 C600</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3652,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>搭载新一代 PH100 芯片的全功能 GPU 智算卡，面向大模型训练、推理与高性能计算；第四代 MUSA「平湖」架构，支持 FP8 到 FP64 全精度 ①</t>
+          <t>沐曦基于自主知识产权 GPGPU 架构与国产先进工艺研发的新一代通用 GPU，面向智算中心、通用计算与数据分析；配 MXMACA 软件栈（兼容主流 GPU 生态）</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3664,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>平湖（第四代 MUSA 架构），含 TCE / TME / ACE 三大引擎 ②</t>
+          <t>自主知识产权 GPGPU 架构（未写代号）</t>
         </is>
       </c>
     </row>
@@ -3179,9 +3674,9 @@
           <t>制程 / 晶体管 / 封装</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>国产先进工艺（未写节点）</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3688,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>OAM 计算模组，液冷版 / 风冷版 ①</t>
+          <t>OAM 2.0 扣卡式模组；风冷 / 液冷</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3700,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>无（官网仅称「超大容量高带宽显存」，支持全链路 ECC）</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3752,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
           <t>FP8 / MXFP8</t>
@@ -3265,7 +3760,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>无（官方只写原生支持 FP8 的 E4M3 / E5M2 格式，未给算力数值）①②</t>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3824,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="34" customHeight="1">
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Scale-up 互连</t>
@@ -3337,7 +3832,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>第二代 MTLink，官方称带宽为上一代 7 倍、支持节点内 8 卡全连接（未给绝对值）②</t>
+          <t>MetaXLink 互连；MetaXLink-E 接口最高 128 卡超节点</t>
         </is>
       </c>
     </row>
@@ -3359,9 +3854,9 @@
           <t>功耗</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>最大功耗 1000W</t>
         </is>
       </c>
     </row>
@@ -3389,15 +3884,15 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="34" customHeight="1">
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>产品页脚注里的 989 TFLOPS / 3.35TB/s 等是对标的「国际旗舰产品」参数，不是 S5000 自身规格 ①</t>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
         </is>
       </c>
     </row>
@@ -3409,21 +3904,8 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>官网产品页：摩尔线程 · MTT S5000
-https://www.mthreads.com/product/S5000</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>来源 ②</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>官网架构页：摩尔线程 ·「平湖」架构
-https://www.mthreads.com/architecture/pinghu</t>
+          <t>官网产品页：沐曦 · 曦云C600
+https://www.metax-tech.com/prod.html?cid=107&amp;id=68</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3916,6 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3446,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3456,7 +3937,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>壁仞 · 官方参数</t>
+          <t>摩尔线程 · 官方参数</t>
         </is>
       </c>
     </row>
@@ -3475,19 +3956,19 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>BR104</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
+          <t>MTT S5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>简介（据官方文档）</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>无：壁仞官网现仅列壁砺 106 / 166 系列；原 BR100 系列页面（birentech.com/BR10X.html）已 404，未见 BR104 官方规格</t>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>搭载新一代 PH100 芯片的全功能 GPU 智算卡，面向大模型训练、推理与高性能计算；第四代 MUSA「平湖」架构，支持 FP8 到 FP64 全精度 ①</t>
         </is>
       </c>
     </row>
@@ -3497,9 +3978,9 @@
           <t>架构</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>平湖（第四代 MUSA 架构），含 TCE / TME / ACE 三大引擎 ②</t>
         </is>
       </c>
     </row>
@@ -3521,9 +4002,9 @@
           <t>形态 / 散热</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>OAM 计算模组，液冷版 / 风冷版 ①</t>
         </is>
       </c>
     </row>
@@ -3587,7 +4068,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
           <t>FP8 / MXFP8</t>
@@ -3595,7 +4076,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>无（官方只写原生支持 FP8 的 E4M3 / E5M2 格式，未给算力数值）①②</t>
         </is>
       </c>
     </row>
@@ -3659,15 +4140,15 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
+    <row r="20" ht="34" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Scale-up 互连</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>第二代 MTLink，官方称带宽为上一代 7 倍、支持节点内 8 卡全连接（未给绝对值）②</t>
         </is>
       </c>
     </row>
@@ -3719,15 +4200,15 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
+    <row r="25" ht="34" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>无</t>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>产品页脚注里的 989 TFLOPS / 3.35TB/s 等是对标的「国际旗舰产品」参数，不是 S5000 自身规格 ①</t>
         </is>
       </c>
     </row>
@@ -3739,8 +4220,21 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>已核查：壁仞官网产品服务（无 BR104）
-https://www.birentech.com/</t>
+          <t>官网产品页：摩尔线程 · MTT S5000
+https://www.mthreads.com/product/S5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>来源 ②</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>官网架构页：摩尔线程 ·「平湖」架构
+https://www.mthreads.com/architecture/pinghu</t>
         </is>
       </c>
     </row>
@@ -3751,6 +4245,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3772,7 +4267,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>海光 · 官方参数</t>
+          <t>壁仞 · 官方参数</t>
         </is>
       </c>
     </row>
@@ -3791,7 +4286,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>DCU3G</t>
+          <t>BR104</t>
         </is>
       </c>
     </row>
@@ -3803,7 +4298,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>无：未找到海光官方公开的 DCU 规格或白皮书</t>
+          <t>无：壁仞官网现仅列壁砺 106 / 166 系列；原 BR100 系列页面（birentech.com/BR10X.html）已 404，未见 BR104 官方规格</t>
         </is>
       </c>
     </row>
@@ -4055,8 +4550,8 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>已核查：海光官网（未见 DCU 规格）
-https://www.hygon.cn/</t>
+          <t>已核查：壁仞官网产品服务（无 BR104）
+https://www.birentech.com/</t>
         </is>
       </c>
     </row>
@@ -4078,6 +4573,322 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>海光 · 官方参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>只收厂商白皮书、datasheet、官网规格页与官方博客 / 文档里写明的数；原文没写的一律填「无」，不换算、不由整机反推单卡；稀疏 / 稠密照原文标注。①②③ 对应表底的来源。核对日期 2026-10-26。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>DCU3G</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>简介（据官方文档）</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>无：未找到海光官方公开的 DCU 规格或白皮书</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>架构</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>制程 / 晶体管 / 封装</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>形态 / 散热</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>显存容量</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>显存类型</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>显存带宽</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>片上 SRAM / 缓存</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>FP4 / MXFP4</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>FP8 / MXFP8</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>BF16 / FP16</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>TF32</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>FP64</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>INT8</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Scale-up 互连</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Scale-out / 主机接口</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>功耗</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>发布 / 上市（官方表述）</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>其他官方指标</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>口径说明</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>来源 ①</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>已核查：海光官网（未见 DCU 规格）
+https://www.hygon.cn/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4402,7 +5213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>